<commit_message>
SEO xlsx: add brand monthly dynamics + peak-index comparison
Динамика по месяцам now shows brand vs non-brand side by side with
index-to-peak columns; brand peaks in April, non-brand in February -
declines are not synchronized.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PUFAzwHkXPjT3b67vFRov4
</commit_message>
<xml_diff>
--- a/yandex-direct/audit/2026-07-19-seo-organic-analysis.xlsx
+++ b/yandex-direct/audit/2026-07-19-seo-organic-analysis.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +50,12 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +70,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,12 +121,16 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -609,59 +622,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Небрендовая органика vs Перегородки-органика, по месяцам</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Бренд vs Небренд vs Перегородки, по месяцам (сравнение падения)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Вся орг. виз</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Бренд виз</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Бренд лиды</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Бренд CR%</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Небренд виз</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Небренд лиды</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Небренд CR%</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Перегородки виз</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Перегородки лиды</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Индекс бренд (пик=100)</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>Индекс небренд (пик=100)</t>
         </is>
       </c>
     </row>
@@ -672,22 +709,34 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>925</v>
+        <v>209</v>
       </c>
       <c r="C4" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.06220095693779904</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>716</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="G4" s="10" t="n">
         <v>0.01256983240223464</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>0</v>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -697,22 +746,34 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>923</v>
+        <v>181</v>
       </c>
       <c r="C5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.04419889502762431</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>742</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="G5" s="10" t="n">
         <v>0.0215633423180593</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>1</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -722,47 +783,71 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1024</v>
+        <v>113</v>
       </c>
       <c r="C6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.01769911504424779</v>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>911</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <v>0.02524698133918771</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="J6" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
-        <v>1383</v>
-      </c>
-      <c r="C7" s="10" t="n">
+      <c r="B7" s="4" t="n">
+        <v>169</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.02366863905325444</v>
+      </c>
+      <c r="E7" s="11" t="n">
         <v>1214</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="F7" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="G7" s="10" t="n">
         <v>0.01812191103789127</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="H7" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="I7" s="4" t="n">
         <v>4</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -772,22 +857,34 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>1011</v>
+        <v>180</v>
       </c>
       <c r="C8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0.04444444444444445</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>831</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>0.01564380264741276</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>2</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="9">
@@ -796,23 +893,35 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>1141</v>
+      <c r="B9" s="12" t="n">
+        <v>394</v>
       </c>
       <c r="C9" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>0.04568527918781726</v>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>747</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <v>0.0214190093708166</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>1</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="10">
@@ -822,22 +931,34 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>851</v>
+        <v>336</v>
       </c>
       <c r="C10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>0.02976190476190476</v>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>515</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="G10" s="10" t="n">
         <v>0.01359223300970874</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="G10" s="4" t="n">
-        <v>0</v>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -847,22 +968,34 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>622</v>
+        <v>170</v>
       </c>
       <c r="C11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>452</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="G11" s="10" t="n">
         <v>0.02876106194690265</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>1</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="12">
@@ -872,28 +1005,54 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>366</v>
+        <v>61</v>
       </c>
       <c r="C12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>0.09836065573770492</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>305</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <v>0.02622950819672131</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="J12" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Февраль - пик небренда (1214), к июлю ~305 (частичный) = минус ~60%</t>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Пики РАЗНЫЕ: небренд пик фев (жёлтый), бренд пик апр (голубой) - падение НЕ синхронно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Небренд: плавный спад с фев (SEO/позиции). Бренд: всплеск апр -&gt; резкий обвал к июлю (событие/сезон).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Июль неполный (до 19-го) - обе серии недосчитаны ~на треть.</t>
         </is>
       </c>
     </row>
@@ -965,216 +1124,216 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>genglass официальный сайт</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="14" t="n">
         <v>437</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="15" t="n">
         <v>0.05491990846681922</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="16" t="n">
         <v>0.0205949657</v>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>genglass</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>333</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="15" t="n">
         <v>0.05405405405405406</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="16" t="n">
         <v>0.015015015</v>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>генгласс</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>107</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.01869158878504673</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="16" t="n">
         <v>0.0280373832</v>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>дженгласс</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="D7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="n">
+      <c r="D7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="n">
         <v>0.0285714286</v>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>genglass официальный</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>58</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.05172413793103448</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="16" t="n">
         <v>0.0862068966</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>генгласс зеркала</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>53</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="15" t="n">
         <v>0.07547169811320754</v>
       </c>
-      <c r="F9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="F9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>дженгласс ру</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="14" t="n">
         <v>52</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="15" t="n">
         <v>0.0576923076923077</v>
       </c>
-      <c r="F10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>gen glass</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="14" t="n">
         <v>44</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="15" t="n">
         <v>0.02272727272727273</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="16" t="n">
         <v>0.0454545455</v>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1195,7 +1354,7 @@
       <c r="D12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
@@ -1218,7 +1377,7 @@
       <c r="D13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -1227,27 +1386,27 @@
       <c r="G13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>genglass.ru</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="14" t="n">
         <v>37</v>
       </c>
-      <c r="D14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="14" t="n">
+      <c r="D14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="16" t="n">
         <v>0.08108108109999999</v>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1268,7 +1427,7 @@
       <c r="D15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>0.03125</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -1291,7 +1450,7 @@
       <c r="D16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -1300,54 +1459,54 @@
       <c r="G16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>ген гласс</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="15" t="n">
         <v>0.03448275862068965</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="16" t="n">
         <v>0.06896551719999999</v>
       </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>генглас</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="15" t="n">
         <v>0.03571428571428571</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F18" s="16" t="n">
         <v>0.1071428571</v>
       </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1368,7 +1527,7 @@
       <c r="D19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -1391,7 +1550,7 @@
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -1414,7 +1573,7 @@
       <c r="D21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="10" t="n">
         <v>0.04</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -1437,7 +1596,7 @@
       <c r="D22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -1460,7 +1619,7 @@
       <c r="D23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="10" t="n">
         <v>0.04761904761904762</v>
       </c>
       <c r="F23" s="5" t="n">
@@ -1469,54 +1628,54 @@
       <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>genglass зеркало</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="D24" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="15" t="n">
         <v>0.05</v>
       </c>
-      <c r="F24" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="F24" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>GENGLASS</t>
         </is>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C25" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="D25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="12" t="inlineStr">
+      <c r="D25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1537,7 +1696,7 @@
       <c r="D26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="9" t="n">
+      <c r="E26" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -1560,7 +1719,7 @@
       <c r="D27" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" s="10" t="n">
         <v>0.05263157894736842</v>
       </c>
       <c r="F27" s="5" t="n">
@@ -1569,81 +1728,81 @@
       <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Genglass</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="D28" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="14" t="n">
+      <c r="D28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="16" t="n">
         <v>0.0625</v>
       </c>
-      <c r="G28" s="12" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n">
+      <c r="A29" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>genglass стол</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n">
+      <c r="C29" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="D29" s="12" t="n">
+      <c r="D29" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="13" t="n">
+      <c r="E29" s="15" t="n">
         <v>0.125</v>
       </c>
-      <c r="F29" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="F29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>стол genglass</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="D30" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="14" t="n">
+      <c r="D30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="16" t="n">
         <v>0.0625</v>
       </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1664,7 +1823,7 @@
       <c r="D31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="9" t="n">
+      <c r="E31" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="5" t="n">
@@ -1687,7 +1846,7 @@
       <c r="D32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="9" t="n">
+      <c r="E32" s="10" t="n">
         <v>0.06666666666666667</v>
       </c>
       <c r="F32" s="5" t="n">
@@ -1696,27 +1855,27 @@
       <c r="G32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n">
+      <c r="A33" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>зеркало genglass</t>
         </is>
       </c>
-      <c r="C33" s="12" t="n">
+      <c r="C33" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="D33" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="D33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1737,7 +1896,7 @@
       <c r="D34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="9" t="n">
+      <c r="E34" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="5" t="n">
@@ -1746,54 +1905,54 @@
       <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="n">
+      <c r="A35" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>купить GENGLASS Зеркало настенное и напольное в полный рост прямоугольное HALFEO Gold XL Slim 200x80 см, ин</t>
         </is>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C35" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="D35" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="12" t="inlineStr">
+      <c r="D35" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n">
+      <c r="A36" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>купить Зеркало напольное в раме GENGLASS Evelum 54х163 см</t>
         </is>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C36" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="13" t="n">
+      <c r="E36" s="15" t="n">
         <v>0.07692307692307693</v>
       </c>
-      <c r="F36" s="14" t="n">
+      <c r="F36" s="16" t="n">
         <v>0.2307692308</v>
       </c>
-      <c r="G36" s="12" t="inlineStr">
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1814,7 +1973,7 @@
       <c r="D37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="9" t="n">
+      <c r="E37" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="5" t="n">
@@ -1823,27 +1982,27 @@
       <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>генгласс столы</t>
         </is>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="D38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="D38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -1864,7 +2023,7 @@
       <c r="D39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="9" t="n">
+      <c r="E39" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="5" t="n">
@@ -1887,7 +2046,7 @@
       <c r="D40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E40" s="9" t="n">
+      <c r="E40" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="5" t="n">
@@ -1910,7 +2069,7 @@
       <c r="D41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E41" s="9" t="n">
+      <c r="E41" s="10" t="n">
         <v>0.09090909090909091</v>
       </c>
       <c r="F41" s="5" t="n">
@@ -1933,7 +2092,7 @@
       <c r="D42" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E42" s="9" t="n">
+      <c r="E42" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="5" t="n">
@@ -1956,7 +2115,7 @@
       <c r="D43" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E43" s="9" t="n">
+      <c r="E43" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="5" t="n">
@@ -1979,7 +2138,7 @@
       <c r="D44" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="9" t="n">
+      <c r="E44" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="5" t="n">
@@ -2002,7 +2161,7 @@
       <c r="D45" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E45" s="9" t="n">
+      <c r="E45" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="5" t="n">
@@ -2025,7 +2184,7 @@
       <c r="D46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E46" s="9" t="n">
+      <c r="E46" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="5" t="n">
@@ -2048,7 +2207,7 @@
       <c r="D47" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E47" s="9" t="n">
+      <c r="E47" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="5" t="n">
@@ -2057,27 +2216,27 @@
       <c r="G47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n">
+      <c r="A48" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>зеркала genglass</t>
         </is>
       </c>
-      <c r="C48" s="12" t="n">
+      <c r="C48" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D48" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="12" t="inlineStr">
+      <c r="D48" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2098,7 +2257,7 @@
       <c r="D49" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E49" s="9" t="n">
+      <c r="E49" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="5" t="n">
@@ -2121,7 +2280,7 @@
       <c r="D50" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E50" s="9" t="n">
+      <c r="E50" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="5" t="n">
@@ -2144,7 +2303,7 @@
       <c r="D51" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="9" t="n">
+      <c r="E51" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F51" s="5" t="n">
@@ -2167,7 +2326,7 @@
       <c r="D52" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="9" t="n">
+      <c r="E52" s="10" t="n">
         <v>0.1111111111111111</v>
       </c>
       <c r="F52" s="5" t="n">
@@ -2176,27 +2335,27 @@
       <c r="G52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="12" t="n">
+      <c r="A53" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>купить GENGLASS Зеркало настенное в полный рост прямоугольное HALFEO Gold XL 200x100 см, интерьерное в золо</t>
         </is>
       </c>
-      <c r="C53" s="12" t="n">
+      <c r="C53" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D53" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="14" t="n">
+      <c r="D53" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="16" t="n">
         <v>0.2222222222</v>
       </c>
-      <c r="G53" s="12" t="inlineStr">
+      <c r="G53" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2217,7 +2376,7 @@
       <c r="D54" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E54" s="9" t="n">
+      <c r="E54" s="10" t="n">
         <v>0.1111111111111111</v>
       </c>
       <c r="F54" s="5" t="n">
@@ -2226,27 +2385,27 @@
       <c r="G54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="n">
+      <c r="A55" s="14" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>настенная стеклянная магнитно-маркерная доска genglass base b-120-240-9003</t>
         </is>
       </c>
-      <c r="C55" s="12" t="n">
+      <c r="C55" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D55" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="12" t="inlineStr">
+      <c r="D55" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2267,7 +2426,7 @@
       <c r="D56" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E56" s="9" t="n">
+      <c r="E56" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F56" s="5" t="n">
@@ -2276,27 +2435,27 @@
       <c r="G56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>genglass зеркало настенное</t>
         </is>
       </c>
-      <c r="C57" s="12" t="n">
+      <c r="C57" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D57" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E57" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F57" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="12" t="inlineStr">
+      <c r="D57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2317,7 +2476,7 @@
       <c r="D58" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="9" t="n">
+      <c r="E58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F58" s="5" t="n">
@@ -2340,7 +2499,7 @@
       <c r="D59" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E59" s="9" t="n">
+      <c r="E59" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F59" s="5" t="n">
@@ -2363,7 +2522,7 @@
       <c r="D60" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E60" s="9" t="n">
+      <c r="E60" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F60" s="5" t="n">
@@ -2386,7 +2545,7 @@
       <c r="D61" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E61" s="9" t="n">
+      <c r="E61" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F61" s="5" t="n">
@@ -2409,7 +2568,7 @@
       <c r="D62" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E62" s="9" t="n">
+      <c r="E62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F62" s="5" t="n">
@@ -2418,27 +2577,27 @@
       <c r="G62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="n">
+      <c r="A63" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="B63" s="12" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>столы genglass</t>
         </is>
       </c>
-      <c r="C63" s="12" t="n">
+      <c r="C63" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D63" s="12" t="n">
+      <c r="D63" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E63" s="13" t="n">
+      <c r="E63" s="15" t="n">
         <v>0.125</v>
       </c>
-      <c r="F63" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" s="12" t="inlineStr">
+      <c r="F63" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2512,189 +2671,189 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>genglass официальный сайт</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="14" t="n">
         <v>318</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="15" t="n">
         <v>0.05031446540880503</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="16" t="n">
         <v>0.0157232704</v>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>genglass</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>245</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="15" t="n">
         <v>0.04081632653061224</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="16" t="n">
         <v>0.012244898</v>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>генгласс</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>78</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.01282051282051282</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="16" t="n">
         <v>0.0384615385</v>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>дженгласс</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>58</v>
       </c>
-      <c r="D7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="n">
+      <c r="D7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="n">
         <v>0.0344827586</v>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>genglass официальный</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="16" t="n">
         <v>0.0666666667</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>генгласс зеркала</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="15" t="n">
         <v>0.08888888888888889</v>
       </c>
-      <c r="F9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="F9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>дженгласс ру</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="14" t="n">
         <v>43</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="15" t="n">
         <v>0.06976744186046512</v>
       </c>
-      <c r="F10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2715,7 +2874,7 @@
       <c r="D11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
@@ -2724,54 +2883,54 @@
       <c r="G11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>gen glass</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="15" t="n">
         <v>0.03703703703703703</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="16" t="n">
         <v>0.0740740741</v>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>genglass.ru</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="D13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="14" t="n">
+      <c r="D13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="16" t="n">
         <v>0.125</v>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2792,7 +2951,7 @@
       <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -2801,27 +2960,27 @@
       <c r="G14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>генглас</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="15" t="n">
         <v>0.04347826086956522</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="16" t="n">
         <v>0.1304347826</v>
       </c>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2842,7 +3001,7 @@
       <c r="D16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -2851,27 +3010,27 @@
       <c r="G16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>ген гласс</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="D17" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="D17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -2892,7 +3051,7 @@
       <c r="D18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="5" t="n">
@@ -2915,7 +3074,7 @@
       <c r="D19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -2938,7 +3097,7 @@
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -2961,7 +3120,7 @@
       <c r="D21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -2984,7 +3143,7 @@
       <c r="D22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -2993,27 +3152,27 @@
       <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>стол genglass</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="D23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="14" t="n">
+      <c r="D23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="16" t="n">
         <v>0.0714285714</v>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3034,7 +3193,7 @@
       <c r="D24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="5" t="n">
@@ -3057,7 +3216,7 @@
       <c r="D25" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="10" t="n">
         <v>0.07692307692307693</v>
       </c>
       <c r="F25" s="5" t="n">
@@ -3066,81 +3225,81 @@
       <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>genglass зеркало</t>
         </is>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D26" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
+      <c r="D26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n">
+      <c r="A27" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>купить GENGLASS Зеркало настенное и напольное в полный рост прямоугольное HALFEO Gold XL Slim 200x80 см, ин</t>
         </is>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C27" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="12" t="inlineStr">
+      <c r="D27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>купить Зеркало напольное в раме GENGLASS Evelum 54х163 см</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D28" s="12" t="n">
+      <c r="D28" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="13" t="n">
+      <c r="E28" s="15" t="n">
         <v>0.08333333333333333</v>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="16" t="n">
         <v>0.1666666667</v>
       </c>
-      <c r="G28" s="12" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3161,7 +3320,7 @@
       <c r="D29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="9" t="n">
+      <c r="E29" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="5" t="n">
@@ -3170,54 +3329,54 @@
       <c r="G29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>GENGLASS</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="D30" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="12" t="inlineStr">
+      <c r="D30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n">
+      <c r="A31" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Genglass</t>
         </is>
       </c>
-      <c r="C31" s="12" t="n">
+      <c r="C31" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="D31" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="14" t="n">
+      <c r="D31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="16" t="n">
         <v>0.0909090909</v>
       </c>
-      <c r="G31" s="12" t="inlineStr">
+      <c r="G31" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3238,7 +3397,7 @@
       <c r="D32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="9" t="n">
+      <c r="E32" s="10" t="n">
         <v>0.09090909090909091</v>
       </c>
       <c r="F32" s="5" t="n">
@@ -3261,7 +3420,7 @@
       <c r="D33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="9" t="n">
+      <c r="E33" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="5" t="n">
@@ -3270,27 +3429,27 @@
       <c r="G33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>зеркало genglass</t>
         </is>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C34" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D34" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="12" t="inlineStr">
+      <c r="D34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3311,7 +3470,7 @@
       <c r="D35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="9" t="n">
+      <c r="E35" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="5" t="n">
@@ -3334,7 +3493,7 @@
       <c r="D36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="9" t="n">
+      <c r="E36" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="5" t="n">
@@ -3357,7 +3516,7 @@
       <c r="D37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="9" t="n">
+      <c r="E37" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="5" t="n">
@@ -3366,27 +3525,27 @@
       <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>генгласс столы</t>
         </is>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="D38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3407,7 +3566,7 @@
       <c r="D39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="9" t="n">
+      <c r="E39" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="5" t="n">
@@ -3416,54 +3575,54 @@
       <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n">
+      <c r="A40" s="14" t="n">
         <v>37</v>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>настенная стеклянная магнитно-маркерная доска genglass base b-120-240-9003</t>
         </is>
       </c>
-      <c r="C40" s="12" t="n">
+      <c r="C40" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D40" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="12" t="inlineStr">
+      <c r="D40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="n">
+      <c r="A41" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>genglass стол</t>
         </is>
       </c>
-      <c r="C41" s="12" t="n">
+      <c r="C41" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D41" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="12" t="inlineStr">
+      <c r="D41" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3484,7 +3643,7 @@
       <c r="D42" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E42" s="9" t="n">
+      <c r="E42" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="5" t="n">
@@ -3493,27 +3652,27 @@
       <c r="G42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="n">
+      <c r="A43" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>зеркала genglass</t>
         </is>
       </c>
-      <c r="C43" s="12" t="n">
+      <c r="C43" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D43" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="12" t="inlineStr">
+      <c r="D43" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3534,7 +3693,7 @@
       <c r="D44" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="9" t="n">
+      <c r="E44" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="5" t="n">
@@ -3557,7 +3716,7 @@
       <c r="D45" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E45" s="9" t="n">
+      <c r="E45" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="5" t="n">
@@ -3566,27 +3725,27 @@
       <c r="G45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="14" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>купить GENGLASS Зеркало настенное в полный рост прямоугольное HALFEO Gold XL 200x100 см, интерьерное в золо</t>
         </is>
       </c>
-      <c r="C46" s="12" t="n">
+      <c r="C46" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D46" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="14" t="n">
+      <c r="D46" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="G46" s="12" t="inlineStr">
+      <c r="G46" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3607,7 +3766,7 @@
       <c r="D47" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="9" t="n">
+      <c r="E47" s="10" t="n">
         <v>0.125</v>
       </c>
       <c r="F47" s="5" t="n">
@@ -3630,7 +3789,7 @@
       <c r="D48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E48" s="9" t="n">
+      <c r="E48" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="5" t="n">
@@ -3653,7 +3812,7 @@
       <c r="D49" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E49" s="9" t="n">
+      <c r="E49" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="5" t="n">
@@ -3676,7 +3835,7 @@
       <c r="D50" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E50" s="9" t="n">
+      <c r="E50" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="5" t="n">
@@ -3699,7 +3858,7 @@
       <c r="D51" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="9" t="n">
+      <c r="E51" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F51" s="5" t="n">
@@ -3722,7 +3881,7 @@
       <c r="D52" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E52" s="9" t="n">
+      <c r="E52" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F52" s="5" t="n">
@@ -3745,7 +3904,7 @@
       <c r="D53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E53" s="9" t="n">
+      <c r="E53" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F53" s="5" t="n">
@@ -3768,7 +3927,7 @@
       <c r="D54" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E54" s="9" t="n">
+      <c r="E54" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F54" s="5" t="n">
@@ -3791,7 +3950,7 @@
       <c r="D55" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E55" s="9" t="n">
+      <c r="E55" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F55" s="5" t="n">
@@ -3814,7 +3973,7 @@
       <c r="D56" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E56" s="9" t="n">
+      <c r="E56" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F56" s="5" t="n">
@@ -3837,7 +3996,7 @@
       <c r="D57" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E57" s="9" t="n">
+      <c r="E57" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="5" t="n">
@@ -3860,7 +4019,7 @@
       <c r="D58" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="9" t="n">
+      <c r="E58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F58" s="5" t="n">
@@ -3883,7 +4042,7 @@
       <c r="D59" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E59" s="9" t="n">
+      <c r="E59" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F59" s="5" t="n">
@@ -3892,27 +4051,27 @@
       <c r="G59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
+      <c r="A60" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>столы genglass</t>
         </is>
       </c>
-      <c r="C60" s="12" t="n">
+      <c r="C60" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="D60" s="12" t="n">
+      <c r="D60" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E60" s="13" t="n">
+      <c r="E60" s="15" t="n">
         <v>0.1666666666666667</v>
       </c>
-      <c r="F60" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="12" t="inlineStr">
+      <c r="F60" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
         <is>
           <t>бренд</t>
         </is>
@@ -3933,7 +4092,7 @@
       <c r="D61" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E61" s="9" t="n">
+      <c r="E61" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F61" s="5" t="n">
@@ -3956,7 +4115,7 @@
       <c r="D62" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E62" s="9" t="n">
+      <c r="E62" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F62" s="5" t="n">
@@ -3979,7 +4138,7 @@
       <c r="D63" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E63" s="9" t="n">
+      <c r="E63" s="10" t="n">
         <v>0.2</v>
       </c>
       <c r="F63" s="5" t="n">

</xml_diff>